<commit_message>
Session 1 complete: model.xlsx scaffold with Cover tab populated
</commit_message>
<xml_diff>
--- a/model.xlsx
+++ b/model.xlsx
@@ -52,7 +52,7 @@
     <t xml:space="preserve">CAD</t>
   </si>
   <si>
-    <t xml:space="preserve">audited</t>
+    <t xml:space="preserve">Historical Window</t>
   </si>
   <si>
     <t xml:space="preserve">FY2021 – FY2025 (audited)</t>
@@ -61,10 +61,10 @@
     <t xml:space="preserve">Forecast Window</t>
   </si>
   <si>
-    <t xml:space="preserve">FY2026 – FY 2030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">primary</t>
+    <t xml:space="preserve">FY2026 – FY2030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valuation Methods</t>
   </si>
   <si>
     <t xml:space="preserve">DCF (primary), Trading Comparables, Scenario Analysis, Monte Carlo</t>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">Source</t>
   </si>
   <si>
-    <t xml:space="preserve">SEDAR+ audited annual financial statements (FY2021-FY2025)</t>
+    <t xml:space="preserve">SEDAR+ audited annual financial statements (FY2021 – FY2025)</t>
   </si>
   <si>
     <t xml:space="preserve">Scope</t>
@@ -103,19 +103,19 @@
     <t xml:space="preserve">Color Legend</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue font</t>
+    <t xml:space="preserve">Blue Font</t>
   </si>
   <si>
     <t xml:space="preserve">Hard-coded input – assumption you can change or historical data</t>
   </si>
   <si>
-    <t xml:space="preserve">Black font</t>
+    <t xml:space="preserve">Black Font</t>
   </si>
   <si>
     <t xml:space="preserve">Formula referencing cells within the same tab</t>
   </si>
   <si>
-    <t xml:space="preserve">Green font</t>
+    <t xml:space="preserve">Green Font</t>
   </si>
   <si>
     <t xml:space="preserve">Formula referencing another tab in this workbook</t>
@@ -124,10 +124,10 @@
     <t xml:space="preserve">Red Font</t>
   </si>
   <si>
-    <t xml:space="preserve">External link to another workbook</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grey fill</t>
+    <t xml:space="preserve">External link to another workbook (avoided – not used here)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grey Fill</t>
   </si>
   <si>
     <t xml:space="preserve">Hardcoded historical actual from audited financial statements</t>
@@ -701,24 +701,22 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="35.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8" t="s">
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="4"/>
+      <c r="C15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="4"/>
+      <c r="C16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="35.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7"/>
+      <c r="B17" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C17" s="9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7"/>

</xml_diff>